<commit_message>
docs: validate CALLAQUI Excel report against manual pivots
</commit_message>
<xml_diff>
--- a/projects/CALLAQUI_PLAN/_EXCEL_OUTPUT/CALLAQUI_INFORME_VALIDACION_GERENCIAL.xlsx
+++ b/projects/CALLAQUI_PLAN/_EXCEL_OUTPUT/CALLAQUI_INFORME_VALIDACION_GERENCIAL.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_LEEME" sheetId="1" r:id="Raf7b5d3d21314d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_RESUMEN" sheetId="2" r:id="Rb5dc3e15a553446f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_PRODUCTIVIDAD_SALA" sheetId="3" r:id="R068071e6b340480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_EVOLUCION_MENSUAL" sheetId="4" r:id="Rf011c9fede134cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_YOY_CONTEXTO" sheetId="5" r:id="Rddd1f750fad04216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ESTABILIDAD" sheetId="6" r:id="R65a1c907671d4f45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OTRAS_ALTO_VOLUMEN" sheetId="7" r:id="Rb3b7fa1d08c74fa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_CONTEXTO_PROMO" sheetId="8" r:id="R34ca01d6b5944888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ANEXOS_TABLAS" sheetId="9" r:id="R08d5f772c05a4bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_QA" sheetId="10" r:id="Rce744a202a184dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_PIVOT_VALIDACION" sheetId="11" r:id="Rf0a172f81c30485f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_LEEME" sheetId="1" r:id="R4841a0485c5c4e59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_RESUMEN" sheetId="2" r:id="R063f5f8da9774845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_PRODUCTIVIDAD_SALA" sheetId="3" r:id="R36c41e170fea4f68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_EVOLUCION_MENSUAL" sheetId="4" r:id="R43a3c3b1f5714b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_YOY_CONTEXTO" sheetId="5" r:id="R3765fa77de5846f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ESTABILIDAD" sheetId="6" r:id="R2b39b48e29d340dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OTRAS_ALTO_VOLUMEN" sheetId="7" r:id="R38554d129ce54a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_CONTEXTO_PROMO" sheetId="8" r:id="Re10fca6dca8b4773"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ANEXOS_TABLAS" sheetId="9" r:id="R4bfddc6a52ee48a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_QA" sheetId="10" r:id="Rc53f85b247704a95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_PIVOT_VALIDACION" sheetId="11" r:id="R6ca5c0ca045e4ce5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,12 +42,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -75,7 +80,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="11">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -102,6 +107,9 @@
     <x:xf numFmtId="204" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -122,8 +130,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="tbl_qa" displayName="tbl_qa" ref="A1:D27" headerRowCount="1">
-  <x:autoFilter ref="A1:D27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_qa" displayName="tbl_qa" ref="A1:D33" headerRowCount="1">
+  <x:autoFilter ref="A1:D33"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="check"/>
     <x:tableColumn id="2" name="estado"/>
@@ -613,7 +621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57d389d6a60249fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R034365365cd545c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -622,23 +630,23 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="46" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="8.25" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="46" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="46" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="10" t="str">
         <x:v>check</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>estado</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>valor</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>detalle</x:v>
       </x:c>
     </x:row>
@@ -754,7 +762,7 @@
         <x:v>Cohorte por percentil 75, sin ranking/top N.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A10" s="2" t="str">
         <x:v>irregularidad_identificador_local</x:v>
       </x:c>
@@ -796,7 +804,7 @@
         <x:v>El encargo pide git push después del commit.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A13" s="2" t="str">
         <x:v>source_final_xlsx</x:v>
       </x:c>
@@ -810,7 +818,7 @@
         <x:v>Fuente obligatoria usada para datos tabulares.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A14" s="2" t="str">
         <x:v>source_final_md</x:v>
       </x:c>
@@ -824,7 +832,7 @@
         <x:v>Fuente obligatoria usada para lectura técnica y contexto.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
+    <x:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A15" s="2" t="str">
         <x:v>hojas_leidas</x:v>
       </x:c>
@@ -894,7 +902,7 @@
         <x:v>Confirmado: junio 2026 llega hasta 21-06-2026.</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="15" hidden="0" customHeight="1">
+    <x:row r="20" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A20" s="2" t="str">
         <x:v>contexto_promocional</x:v>
       </x:c>
@@ -927,30 +935,30 @@
         <x:v>VALIDACION_MANUAL_REVISADA</x:v>
       </x:c>
       <x:c r="B22" s="2" t="str">
-        <x:v>INFO</x:v>
+        <x:v>OK</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
-        <x:v>NO</x:v>
+        <x:v>SI</x:v>
       </x:c>
       <x:c r="D22" s="2" t="str">
-        <x:v>No se abrió el Excel original; no hubo inconsistencia crítica que justificara revisarlo.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="15" hidden="0" customHeight="1">
+        <x:v>Hoja DINAMICA revisada en modo lectura; las dinámicas visibles usan Suma de Vta_KG.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A23" s="2" t="str">
         <x:v>ARCHIVO_VALIDACION_MANUAL</x:v>
       </x:c>
       <x:c r="B23" s="2" t="str">
-        <x:v>INFO</x:v>
+        <x:v>OK</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
         <x:v>projects/CALLAQUI_PLAN/Callaqui 2025-2026.xlsx</x:v>
       </x:c>
       <x:c r="D23" s="2" t="str">
-        <x:v>Archivo original disponible solo para contraste manual posterior.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="15" hidden="0" customHeight="1">
+        <x:v>Archivo original usado solo lectura; no se guardó ni modificó.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A24" s="2" t="str">
         <x:v>ORIGINAL_WORKBOOK_MODIFIED_DURANTE_TAREA</x:v>
       </x:c>
@@ -961,7 +969,7 @@
         <x:v>NO</x:v>
       </x:c>
       <x:c r="D24" s="2" t="str">
-        <x:v>La generación no modificó el workbook original.</x:v>
+        <x:v>Hash y estado Git se validan antes/después; el original no fue modificado.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
@@ -1006,10 +1014,94 @@
         <x:v>Últimos tres commits registrados antes de generar el archivo.</x:v>
       </x:c>
     </x:row>
+    <x:row r="28" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A28" s="2" t="str">
+        <x:v>VALIDACION_MANUAL_RESULTADO</x:v>
+      </x:c>
+      <x:c r="B28" s="2" t="str">
+        <x:v>WARN</x:v>
+      </x:c>
+      <x:c r="C28" s="2" t="str">
+        <x:v>NO_CUADRA</x:v>
+      </x:c>
+      <x:c r="D28" s="2" t="str">
+        <x:v>RT en kg cuadra con DINAMICA; OTRAS kg difiere contra pivotes visibles y no hay venta público visible en dinámicas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A29" s="2" t="str">
+        <x:v>DIFERENCIAS_DETECTADAS</x:v>
+      </x:c>
+      <x:c r="B29" s="2" t="str">
+        <x:v>WARN</x:v>
+      </x:c>
+      <x:c r="C29" s="2" t="str">
+        <x:v>OTRAS kg manual menor; venta no visible</x:v>
+      </x:c>
+      <x:c r="D29" s="2" t="str">
+        <x:v>OTRAS kg DINAMICA vs analítico: 2025 23.029,50 vs 25.920,02; 2026 25.900,69 vs 28.593,75. Mayo/junio OTRAS también menor. Venta público no aparece como valor en pivotes guardados.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="15" hidden="0" customHeight="1">
+      <x:c r="A30" s="2" t="str">
+        <x:v>DINAMICAS_MANUALES_REVISADAS</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>DINAMICA</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>9 tablas dinámicas guardadas; campo de valor detectado: Suma de Vta_KG.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>KG_RT_VALIDACION</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>CUADRA</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>RT kg: 2025 3.956,53 y 2026 3.820,76; mayo 2025, mayo 2026 y junio 2026 coinciden con analítico.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>KG_OTRAS_VALIDACION</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>WARN</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>NO_CUADRA</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>OTRAS kg en dinámicas visibles queda 9%-11% bajo el analítico final; probable diferencia de filtros/universo manual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A33" s="2" t="str">
+        <x:v>VENTA_PUBLICO_EN_DINAMICAS</x:v>
+      </x:c>
+      <x:c r="B33" s="2" t="str">
+        <x:v>WARN</x:v>
+      </x:c>
+      <x:c r="C33" s="2" t="str">
+        <x:v>NO_VISIBLE</x:v>
+      </x:c>
+      <x:c r="D33" s="2" t="str">
+        <x:v>La metadata de 9 pivotes muestra solo Suma de Vta_KG como campo de valor; no se validó venta público contra dinámica manual.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0385b1648de9427f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R158da6acb3e84ac1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3449,7 +3541,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a78f3e209fd40e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra23226a3818b4e50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3703,7 +3795,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R854ed2a78fde4195"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb41d0f557e8c4f8c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3871,7 +3963,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f910b4faea240c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refaa40e796264714"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4847,7 +4939,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71180cd03f8a46d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5180049cb7af4589"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4947,7 +5039,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17290830630047e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74b1dc1c15484859"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5037,7 +5129,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reab56af901324b61"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra56399b5bb0b40e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5125,7 +5217,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6121500b85364657"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R407553a735234f39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5208,7 +5300,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38a52dadc76d40a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9208943413584219"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5302,7 +5394,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbea36d3ac0104a60"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f091f2c3784efd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
qa: reconcile CALLAQUI OTRAS kg against manual pivots
</commit_message>
<xml_diff>
--- a/projects/CALLAQUI_PLAN/_EXCEL_OUTPUT/CALLAQUI_INFORME_VALIDACION_GERENCIAL.xlsx
+++ b/projects/CALLAQUI_PLAN/_EXCEL_OUTPUT/CALLAQUI_INFORME_VALIDACION_GERENCIAL.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_LEEME" sheetId="1" r:id="R4841a0485c5c4e59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_RESUMEN" sheetId="2" r:id="R063f5f8da9774845"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_PRODUCTIVIDAD_SALA" sheetId="3" r:id="R36c41e170fea4f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_EVOLUCION_MENSUAL" sheetId="4" r:id="R43a3c3b1f5714b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_YOY_CONTEXTO" sheetId="5" r:id="R3765fa77de5846f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ESTABILIDAD" sheetId="6" r:id="R2b39b48e29d340dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OTRAS_ALTO_VOLUMEN" sheetId="7" r:id="R38554d129ce54a22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_CONTEXTO_PROMO" sheetId="8" r:id="Re10fca6dca8b4773"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ANEXOS_TABLAS" sheetId="9" r:id="R4bfddc6a52ee48a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_QA" sheetId="10" r:id="Rc53f85b247704a95"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_PIVOT_VALIDACION" sheetId="11" r:id="R6ca5c0ca045e4ce5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_LEEME" sheetId="1" r:id="Ra95da9c94e3f488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_RESUMEN" sheetId="2" r:id="Rc016b6b15b744f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_PRODUCTIVIDAD_SALA" sheetId="3" r:id="Ra19804bce55b4eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_EVOLUCION_MENSUAL" sheetId="4" r:id="R1e962ee5b5f74614"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_YOY_CONTEXTO" sheetId="5" r:id="R01c9c07706d3452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_ESTABILIDAD" sheetId="6" r:id="R0d5374be5ba1459d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_OTRAS_ALTO_VOLUMEN" sheetId="7" r:id="Rbee36a1c2bd8452d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_CONTEXTO_PROMO" sheetId="8" r:id="R4719d346a9de4bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_ANEXOS_TABLAS" sheetId="9" r:id="Re4ff065ef9964dd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_QA" sheetId="10" r:id="Rdedeacc135ac4c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_PIVOT_VALIDACION" sheetId="11" r:id="R3e922ca29c6f493c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,12 +42,17 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -80,7 +85,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="12">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -110,6 +115,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -130,8 +138,8 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_qa" displayName="tbl_qa" ref="A1:D33" headerRowCount="1">
-  <x:autoFilter ref="A1:D33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tbl_qa" displayName="tbl_qa" ref="A1:D37" headerRowCount="1">
+  <x:autoFilter ref="A1:D37"/>
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="check"/>
     <x:tableColumn id="2" name="estado"/>
@@ -621,7 +629,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R034365365cd545c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf11d76fa538e4a00"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -632,21 +640,21 @@
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="68" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="76" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
-      <x:c r="A1" s="10" t="str">
+      <x:c r="A1" s="11" t="str">
         <x:v>check</x:v>
       </x:c>
-      <x:c r="B1" s="10" t="str">
+      <x:c r="B1" s="11" t="str">
         <x:v>estado</x:v>
       </x:c>
-      <x:c r="C1" s="10" t="str">
+      <x:c r="C1" s="11" t="str">
         <x:v>valor</x:v>
       </x:c>
-      <x:c r="D1" s="10" t="str">
+      <x:c r="D1" s="11" t="str">
         <x:v>detalle</x:v>
       </x:c>
     </x:row>
@@ -762,7 +770,7 @@
         <x:v>Cohorte por percentil 75, sin ranking/top N.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="2" t="str">
         <x:v>irregularidad_identificador_local</x:v>
       </x:c>
@@ -818,7 +826,7 @@
         <x:v>Fuente obligatoria usada para datos tabulares.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A14" s="2" t="str">
         <x:v>source_final_md</x:v>
       </x:c>
@@ -832,7 +840,7 @@
         <x:v>Fuente obligatoria usada para lectura técnica y contexto.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="92.4000015258789" hidden="0" customHeight="1">
+    <x:row r="15" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A15" s="2" t="str">
         <x:v>hojas_leidas</x:v>
       </x:c>
@@ -944,7 +952,7 @@
         <x:v>Hoja DINAMICA revisada en modo lectura; las dinámicas visibles usan Suma de Vta_KG.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="2" t="str">
         <x:v>ARCHIVO_VALIDACION_MANUAL</x:v>
       </x:c>
@@ -1022,24 +1030,24 @@
         <x:v>WARN</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
-        <x:v>NO_CUADRA</x:v>
+        <x:v>CUADRA_PARCIAL</x:v>
       </x:c>
       <x:c r="D28" s="2" t="str">
-        <x:v>RT en kg cuadra con DINAMICA; OTRAS kg difiere contra pivotes visibles y no hay venta público visible en dinámicas.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="39.599998474121094" hidden="0" customHeight="1">
+        <x:v>RT cuadra; OTRAS no cuadra contra dinámica visible, pero la diferencia queda explicada por filtro FORMATO.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A29" s="2" t="str">
         <x:v>DIFERENCIAS_DETECTADAS</x:v>
       </x:c>
       <x:c r="B29" s="2" t="str">
-        <x:v>WARN</x:v>
+        <x:v>OK</x:v>
       </x:c>
       <x:c r="C29" s="2" t="str">
-        <x:v>OTRAS kg manual menor; venta no visible</x:v>
+        <x:v>Diferencia explicada por FORMATO</x:v>
       </x:c>
       <x:c r="D29" s="2" t="str">
-        <x:v>OTRAS kg DINAMICA vs analítico: 2025 23.029,50 vs 25.920,02; 2026 25.900,69 vs 28.593,75. Mayo/junio OTRAS también menor. Venta público no aparece como valor en pivotes guardados.</x:v>
+        <x:v>OTRAS dinámica manual oculta CONVENIENCIA y SANTA ISABEL; esos kg explican la brecha contra el analítico final.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
@@ -1056,7 +1064,7 @@
         <x:v>9 tablas dinámicas guardadas; campo de valor detectado: Suma de Vta_KG.</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="2" t="str">
         <x:v>KG_RT_VALIDACION</x:v>
       </x:c>
@@ -1070,7 +1078,7 @@
         <x:v>RT kg: 2025 3.956,53 y 2026 3.820,76; mayo 2025, mayo 2026 y junio 2026 coinciden con analítico.</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="2" t="str">
         <x:v>KG_OTRAS_VALIDACION</x:v>
       </x:c>
@@ -1078,10 +1086,10 @@
         <x:v>WARN</x:v>
       </x:c>
       <x:c r="C32" s="2" t="str">
-        <x:v>NO_CUADRA</x:v>
+        <x:v>CUADRA_PARCIAL</x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
-        <x:v>OTRAS kg en dinámicas visibles queda 9%-11% bajo el analítico final; probable diferencia de filtros/universo manual.</x:v>
+        <x:v>No cuadra contra total analítico sin filtro; cuadra al aplicar FORMATO in JUMBO,JUMBO MARKET.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1098,10 +1106,66 @@
         <x:v>La metadata de 9 pivotes muestra solo Suma de Vta_KG como campo de valor; no se validó venta público contra dinámica manual.</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" ht="15" hidden="0" customHeight="1">
+      <x:c r="A34" s="2" t="str">
+        <x:v>CONCILIACION_OTRAS_KG_REALIZADA</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>SI</x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>Conciliación documentada en _QA_OUTPUT/CALLAQUI_CONCILIACION_OTRAS_KG.md y .xlsx.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A35" s="2" t="str">
+        <x:v>CONCILIACION_OTRAS_KG_RESULTADO</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>DIFERENCIA_EXPLICADA_POR_FILTROS</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>Filtros manuales visibles: FORMATO=JUMBO/JUMBO MARKET; ocultos: CONVENIENCIA/SANTA ISABEL.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="15" hidden="0" customHeight="1">
+      <x:c r="A36" s="2" t="str">
+        <x:v>FUENTE_CANONICA_PDF</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>ANALITICO_FINAL</x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>Usar si el PDF mantiene el universo completo; declarar alcance frente a dinámicas manuales.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A37" s="2" t="str">
+        <x:v>OBSERVACION_OTRAS_KG</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="str">
+        <x:v>OK</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>OTRAS manual es vista parcial por FORMATO</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="str">
+        <x:v>La diferencia total 2025-2026 de -5.583,58 kg coincide con kg excluido por CONVENIENCIA y SANTA ISABEL.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R158da6acb3e84ac1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R378437b3198a4f02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3541,7 +3605,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra23226a3818b4e50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ef04ab7f8124f19"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3795,7 +3859,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb41d0f557e8c4f8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fae23f2e96544fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3963,7 +4027,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refaa40e796264714"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39c02b15bea74977"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4939,7 +5003,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5180049cb7af4589"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2625d04e69ae408c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5039,7 +5103,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74b1dc1c15484859"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8edd546fd4d4390"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5129,7 +5193,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra56399b5bb0b40e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0d8e9ac02064b20"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5217,7 +5281,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R407553a735234f39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f2adae7012943b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5300,7 +5364,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9208943413584219"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21b9a714af44518"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5394,7 +5458,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10f091f2c3784efd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85683ad6509848bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>